<commit_message>
Foso: columnas con 4 #4 y fleje #3 L=1.48 m
Actualiza la cartilla, el cuadro de cantidades, la memoria y los esquemas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGm1Wo5xdbH6HEAejZfCqA
</commit_message>
<xml_diff>
--- a/cantidades/Cantidades_Multifamiliar_Herrera.xlsx
+++ b/cantidades/Cantidades_Multifamiliar_Herrera.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="730" uniqueCount="489">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="727" uniqueCount="489">
   <si>
     <t xml:space="preserve">RESUMEN DE CANTIDADES PRINCIPALES — MULTIFAMILIAR HERRERA</t>
   </si>
@@ -261,7 +261,7 @@
     <t xml:space="preserve">Acero de refuerzo #4 (1/2")</t>
   </si>
   <si>
-    <t xml:space="preserve">Acero corrugado fy = 420 MPa (60.000 psi), NTC 2289. Losa doble parrilla #4 c/0.20; muros #4 c/0.20 en ambos sentidos; longitudinal de columnas. Figurado según cartilla (hoja Foso ascensor).</t>
+    <t xml:space="preserve">Acero corrugado fy = 420 MPa (60.000 psi), NTC 2289. Losa doble parrilla #4 c/0.20; muros #4 c/0.20 en ambos sentidos; longitudinal de columnas 4 #4 por columna. Figurado según cartilla (hoja Foso ascensor).</t>
   </si>
   <si>
     <t xml:space="preserve">2.7</t>
@@ -270,7 +270,7 @@
     <t xml:space="preserve">Acero de refuerzo #3 (3/8") — flejes</t>
   </si>
   <si>
-    <t xml:space="preserve">Acero corrugado fy = 420 MPa, NTC 2289. Flejes cerrados #3 @0.075 m, gancho a 135°.</t>
+    <t xml:space="preserve">Acero corrugado fy = 420 MPa, NTC 2289. Flejes cerrados #3 @0.075 m, L = 1.48 m, gancho a 135°.</t>
   </si>
   <si>
     <t xml:space="preserve">2.8</t>
@@ -1329,10 +1329,7 @@
     <t xml:space="preserve">Columnas 40×40 — longitudinal</t>
   </si>
   <si>
-    <t xml:space="preserve">Detalle sección columna: 6 #4 L=1.80</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Detalle sección columna: 6 #4 L=1.85</t>
+    <t xml:space="preserve">Confirmado: 4 #4 por columna (L=1.85 del detalle)</t>
   </si>
   <si>
     <t xml:space="preserve">Columnas 40×40 — flejes cerrados</t>
@@ -1341,7 +1338,7 @@
     <t xml:space="preserve">#3</t>
   </si>
   <si>
-    <t xml:space="preserve">Detalle columna: fleje #3 @0.075 L=1.50</t>
+    <t xml:space="preserve">Confirmado: fleje #3 @0.075 L=1.48</t>
   </si>
   <si>
     <t xml:space="preserve">Subtotal #4 (sin desperdicio)</t>
@@ -1437,19 +1434,22 @@
     <t xml:space="preserve">Coordinar la ubicación del ducto en planta arquitectónica y la ficha del proveedor (foso útil 1.20 m, luz 1.50 × 1.90 m).</t>
   </si>
   <si>
+    <t xml:space="preserve">Resuelto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Columnas 40×40: confirmado 4 #4 por columna (16 barras en total). Se tomó L=1.85 m del detalle de refuerzo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmado por el arquitecto. Verificar que la longitud de 1.85 m quede en la cartilla final.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flejes: confirmado fleje #3 @0.075 con L=1.48 m (80 flejes en total).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmado por el arquitecto.</t>
+  </si>
+  <si>
     <t xml:space="preserve">EST-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Columnas 40×40: la sección muestra 4 #4, pero el detalle de refuerzo indica 6 #4 L=1.80 + 6 #4 L=1.85. Se cuantificaron ambas tandas (12 barras por columna).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirmar con el calculista (Ing. A. Trujillo Rivas). Si es solo 4 #4, el acero #4 baja ≈ 60 kg.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flejes: aparecen dos longitudes (L=1.50 m y L=1.90 m) para el fleje #3 @0.075. Se usó L=1.50 m.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirmar. Con L=1.90 m el acero #3 sube ≈ 18 kg.</t>
   </si>
   <si>
     <t xml:space="preserve">Barras de losa: la planta indica L=2.10/2.50 y los cortes L=2.20/2.60. Se usaron las de los cortes (losa) y las de planta (horizontales de muros).</t>
@@ -2329,8 +2329,8 @@
         <v>24</v>
       </c>
       <c r="B13" s="6" t="n">
-        <f aca="false">('Foso ascensor'!K54+'Foso ascensor'!K55)*(1+Supuestos!$B$6)</f>
-        <v>404.33526</v>
+        <f aca="false">('Foso ascensor'!K53+'Foso ascensor'!K54)*(1+Supuestos!$B$6)</f>
+        <v>342.85986</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>25</v>
@@ -2702,7 +2702,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
         <v>75</v>
       </c>
@@ -2721,8 +2721,8 @@
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
       <c r="J14" s="10" t="n">
-        <f aca="false">'Foso ascensor'!K54*(1+Supuestos!$B$6)</f>
-        <v>333.77526</v>
+        <f aca="false">'Foso ascensor'!K53*(1+Supuestos!$B$6)</f>
+        <v>273.24066</v>
       </c>
       <c r="K14" s="11" t="s">
         <v>58</v>
@@ -2750,8 +2750,8 @@
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
       <c r="J15" s="10" t="n">
-        <f aca="false">'Foso ascensor'!K55*(1+Supuestos!$B$6)</f>
-        <v>70.56</v>
+        <f aca="false">'Foso ascensor'!K54*(1+Supuestos!$B$6)</f>
+        <v>69.6192</v>
       </c>
       <c r="K15" s="11" t="s">
         <v>58</v>
@@ -2891,7 +2891,7 @@
       <c r="H20" s="5"/>
       <c r="I20" s="5"/>
       <c r="J20" s="13" t="n">
-        <f aca="false">'Foso ascensor'!B60</f>
+        <f aca="false">'Foso ascensor'!B59</f>
         <v>4</v>
       </c>
       <c r="K20" s="11" t="s">
@@ -2920,7 +2920,7 @@
       <c r="H21" s="5"/>
       <c r="I21" s="5"/>
       <c r="J21" s="13" t="n">
-        <f aca="false">'Foso ascensor'!B62</f>
+        <f aca="false">'Foso ascensor'!B61</f>
         <v>16</v>
       </c>
       <c r="K21" s="11" t="s">
@@ -2947,7 +2947,7 @@
       <c r="H22" s="5"/>
       <c r="I22" s="5"/>
       <c r="J22" s="10" t="n">
-        <f aca="false">'Foso ascensor'!B63</f>
+        <f aca="false">'Foso ascensor'!B62</f>
         <v>4.6</v>
       </c>
       <c r="K22" s="11" t="s">
@@ -2976,7 +2976,7 @@
       <c r="H23" s="5"/>
       <c r="I23" s="5"/>
       <c r="J23" s="13" t="n">
-        <f aca="false">'Foso ascensor'!B64</f>
+        <f aca="false">'Foso ascensor'!B63</f>
         <v>4</v>
       </c>
       <c r="K23" s="11" t="s">
@@ -6343,7 +6343,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L63"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -7552,21 +7552,21 @@
       <c r="C51" s="32"/>
       <c r="D51" s="31"/>
       <c r="E51" s="25" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F51" s="25" t="n">
         <v>4</v>
       </c>
       <c r="G51" s="37" t="n">
         <f aca="false">E51*F51</f>
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="H51" s="29" t="n">
-        <v>1.8</v>
+        <v>1.85</v>
       </c>
       <c r="I51" s="18" t="n">
         <f aca="false">G51*H51</f>
-        <v>43.2</v>
+        <v>29.6</v>
       </c>
       <c r="J51" s="38" t="n">
         <f aca="false">Supuestos!$B$5</f>
@@ -7574,7 +7574,7 @@
       </c>
       <c r="K51" s="18" t="n">
         <f aca="false">I51*J51</f>
-        <v>42.9408</v>
+        <v>29.4224</v>
       </c>
       <c r="L51" s="5" t="s">
         <v>433</v>
@@ -7582,85 +7582,69 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>421</v>
-      </c>
-      <c r="C52" s="32"/>
-      <c r="D52" s="31"/>
-      <c r="E52" s="25" t="n">
-        <v>6</v>
+        <v>435</v>
+      </c>
+      <c r="C52" s="26" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="D52" s="31" t="n">
+        <f aca="false">$B$13</f>
+        <v>1.4</v>
+      </c>
+      <c r="E52" s="37" t="n">
+        <f aca="false">ROUNDUP(D52/C52,0)+1</f>
+        <v>20</v>
       </c>
       <c r="F52" s="25" t="n">
         <v>4</v>
       </c>
       <c r="G52" s="37" t="n">
         <f aca="false">E52*F52</f>
-        <v>24</v>
+        <v>80</v>
       </c>
       <c r="H52" s="29" t="n">
-        <v>1.85</v>
+        <v>1.48</v>
       </c>
       <c r="I52" s="18" t="n">
         <f aca="false">G52*H52</f>
-        <v>44.4</v>
+        <v>118.4</v>
       </c>
       <c r="J52" s="38" t="n">
-        <f aca="false">Supuestos!$B$5</f>
-        <v>0.994</v>
+        <f aca="false">Supuestos!$B$4</f>
+        <v>0.56</v>
       </c>
       <c r="K52" s="18" t="n">
         <f aca="false">I52*J52</f>
-        <v>44.1336</v>
+        <v>66.304</v>
       </c>
       <c r="L52" s="5" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="5" t="s">
-        <v>435</v>
-      </c>
-      <c r="B53" s="5" t="s">
-        <v>436</v>
-      </c>
-      <c r="C53" s="26" t="n">
-        <v>0.075</v>
-      </c>
-      <c r="D53" s="31" t="n">
-        <f aca="false">$B$13</f>
-        <v>1.4</v>
-      </c>
-      <c r="E53" s="37" t="n">
-        <f aca="false">ROUNDUP(D53/C53,0)+1</f>
-        <v>20</v>
-      </c>
-      <c r="F53" s="25" t="n">
-        <v>4</v>
-      </c>
-      <c r="G53" s="37" t="n">
-        <f aca="false">E53*F53</f>
-        <v>80</v>
-      </c>
-      <c r="H53" s="29" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="I53" s="18" t="n">
-        <f aca="false">G53*H53</f>
-        <v>120</v>
-      </c>
-      <c r="J53" s="38" t="n">
-        <f aca="false">Supuestos!$B$4</f>
-        <v>0.56</v>
-      </c>
-      <c r="K53" s="18" t="n">
-        <f aca="false">I53*J53</f>
-        <v>67.2</v>
-      </c>
-      <c r="L53" s="5" t="s">
+      <c r="A53" s="27" t="s">
         <v>437</v>
       </c>
+      <c r="B53" s="2"/>
+      <c r="C53" s="2"/>
+      <c r="D53" s="2"/>
+      <c r="E53" s="2"/>
+      <c r="F53" s="2"/>
+      <c r="G53" s="2"/>
+      <c r="H53" s="2"/>
+      <c r="I53" s="36" t="n">
+        <f aca="false">SUMIF(B45:B52,"#4",I45:I52)</f>
+        <v>261.8</v>
+      </c>
+      <c r="J53" s="2"/>
+      <c r="K53" s="36" t="n">
+        <f aca="false">SUMIF(B45:B52,"#4",K45:K52)</f>
+        <v>260.2292</v>
+      </c>
+      <c r="L53" s="2"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="27" t="s">
@@ -7674,18 +7658,18 @@
       <c r="G54" s="2"/>
       <c r="H54" s="2"/>
       <c r="I54" s="36" t="n">
-        <f aca="false">SUMIF(B45:B53,"#4",I45:I53)</f>
-        <v>319.8</v>
+        <f aca="false">SUMIF(B45:B52,"#3",I45:I52)</f>
+        <v>118.4</v>
       </c>
       <c r="J54" s="2"/>
       <c r="K54" s="36" t="n">
-        <f aca="false">SUMIF(B45:B53,"#4",K45:K53)</f>
-        <v>317.8812</v>
+        <f aca="false">SUMIF(B45:B52,"#3",K45:K52)</f>
+        <v>66.304</v>
       </c>
       <c r="L54" s="2"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="27" t="s">
+      <c r="A55" s="39" t="s">
         <v>439</v>
       </c>
       <c r="B55" s="2"/>
@@ -7695,21 +7679,16 @@
       <c r="F55" s="2"/>
       <c r="G55" s="2"/>
       <c r="H55" s="2"/>
-      <c r="I55" s="36" t="n">
-        <f aca="false">SUMIF(B45:B53,"#3",I45:I53)</f>
-        <v>120</v>
-      </c>
+      <c r="I55" s="2"/>
       <c r="J55" s="2"/>
-      <c r="K55" s="36" t="n">
-        <f aca="false">SUMIF(B45:B53,"#3",K45:K53)</f>
-        <v>67.2</v>
+      <c r="K55" s="40" t="n">
+        <f aca="false">(K53+K54)/B29</f>
+        <v>120.137306843267</v>
       </c>
       <c r="L55" s="2"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="39" t="s">
-        <v>440</v>
-      </c>
+      <c r="A56" s="2"/>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
@@ -7719,14 +7698,13 @@
       <c r="H56" s="2"/>
       <c r="I56" s="2"/>
       <c r="J56" s="2"/>
-      <c r="K56" s="40" t="n">
-        <f aca="false">(K54+K55)/B29</f>
-        <v>141.678145695364</v>
-      </c>
+      <c r="K56" s="2"/>
       <c r="L56" s="2"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="2"/>
+      <c r="A57" s="23" t="s">
+        <v>440</v>
+      </c>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
@@ -7739,13 +7717,19 @@
       <c r="K57" s="2"/>
       <c r="L57" s="2"/>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="23" t="s">
+    <row r="58" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="D58" s="4" t="s">
         <v>441</v>
       </c>
-      <c r="B58" s="2"/>
-      <c r="C58" s="2"/>
-      <c r="D58" s="2"/>
       <c r="E58" s="2"/>
       <c r="F58" s="2"/>
       <c r="G58" s="2"/>
@@ -7755,18 +7739,19 @@
       <c r="K58" s="2"/>
       <c r="L58" s="2"/>
     </row>
-    <row r="59" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="4" t="s">
-        <v>378</v>
-      </c>
-      <c r="B59" s="4" t="s">
-        <v>379</v>
-      </c>
-      <c r="C59" s="4" t="s">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="5" t="s">
+        <v>442</v>
+      </c>
+      <c r="B59" s="37" t="n">
+        <f aca="false">$B$10</f>
         <v>4</v>
       </c>
-      <c r="D59" s="4" t="s">
-        <v>442</v>
+      <c r="C59" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D59" s="5" t="s">
+        <v>443</v>
       </c>
       <c r="E59" s="2"/>
       <c r="F59" s="2"/>
@@ -7777,19 +7762,19 @@
       <c r="K59" s="2"/>
       <c r="L59" s="2"/>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
-        <v>443</v>
-      </c>
-      <c r="B60" s="37" t="n">
-        <f aca="false">$B$10</f>
-        <v>4</v>
+        <v>444</v>
+      </c>
+      <c r="B60" s="18" t="n">
+        <f aca="false">B59*0.3*0.3*0.016*Supuestos!$B$18</f>
+        <v>45.216</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E60" s="2"/>
       <c r="F60" s="2"/>
@@ -7800,16 +7785,16 @@
       <c r="K60" s="2"/>
       <c r="L60" s="2"/>
     </row>
-    <row r="61" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
-        <v>445</v>
-      </c>
-      <c r="B61" s="18" t="n">
-        <f aca="false">B60*0.3*0.3*0.016*Supuestos!$B$18</f>
-        <v>45.216</v>
+        <v>101</v>
+      </c>
+      <c r="B61" s="37" t="n">
+        <f aca="false">4*$B$10</f>
+        <v>16</v>
       </c>
       <c r="C61" s="5" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D61" s="5" t="s">
         <v>446</v>
@@ -7823,19 +7808,19 @@
       <c r="K61" s="2"/>
       <c r="L61" s="2"/>
     </row>
-    <row r="62" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="B62" s="37" t="n">
-        <f aca="false">4*$B$10</f>
-        <v>16</v>
+        <v>447</v>
+      </c>
+      <c r="B62" s="18" t="n">
+        <f aca="false">$B$10*1.15</f>
+        <v>4.6</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>15</v>
+        <v>106</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E62" s="2"/>
       <c r="F62" s="2"/>
@@ -7846,19 +7831,19 @@
       <c r="K62" s="2"/>
       <c r="L62" s="2"/>
     </row>
-    <row r="63" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="s">
-        <v>448</v>
-      </c>
-      <c r="B63" s="18" t="n">
-        <f aca="false">$B$10*1.15</f>
-        <v>4.6</v>
+        <v>449</v>
+      </c>
+      <c r="B63" s="37" t="n">
+        <f aca="false">$B$10</f>
+        <v>4</v>
       </c>
       <c r="C63" s="5" t="s">
-        <v>106</v>
+        <v>15</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="E63" s="2"/>
       <c r="F63" s="2"/>
@@ -7868,29 +7853,6 @@
       <c r="J63" s="2"/>
       <c r="K63" s="2"/>
       <c r="L63" s="2"/>
-    </row>
-    <row r="64" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="5" t="s">
-        <v>450</v>
-      </c>
-      <c r="B64" s="37" t="n">
-        <f aca="false">$B$10</f>
-        <v>4</v>
-      </c>
-      <c r="C64" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D64" s="5" t="s">
-        <v>451</v>
-      </c>
-      <c r="E64" s="2"/>
-      <c r="F64" s="2"/>
-      <c r="G64" s="2"/>
-      <c r="H64" s="2"/>
-      <c r="I64" s="2"/>
-      <c r="J64" s="2"/>
-      <c r="K64" s="2"/>
-      <c r="L64" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -7919,7 +7881,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -7933,16 +7895,16 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
+        <v>452</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>453</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="C3" s="4" t="s">
         <v>454</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>455</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>456</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7950,13 +7912,13 @@
         <v>1</v>
       </c>
       <c r="B4" s="5" t="s">
+        <v>456</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>457</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>458</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>459</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7964,13 +7926,13 @@
         <v>2</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="C5" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>460</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>461</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7978,13 +7940,13 @@
         <v>3</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="C6" s="5" t="s">
+        <v>461</v>
+      </c>
+      <c r="D6" s="5" t="s">
         <v>462</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>463</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7992,13 +7954,13 @@
         <v>4</v>
       </c>
       <c r="B7" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>464</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="D7" s="5" t="s">
         <v>465</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>466</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8006,13 +7968,13 @@
         <v>5</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="C8" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>467</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>468</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8020,13 +7982,13 @@
         <v>6</v>
       </c>
       <c r="B9" s="5" t="s">
+        <v>468</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>469</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="D9" s="5" t="s">
         <v>470</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>471</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8034,13 +7996,13 @@
         <v>7</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="C10" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>472</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>473</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8048,7 +8010,7 @@
         <v>8</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>474</v>
@@ -8062,7 +8024,7 @@
         <v>9</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>476</v>
@@ -8076,7 +8038,7 @@
         <v>10</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>478</v>

</xml_diff>

<commit_message>
Foso: varillas de columna con longitud total de 1.80 m
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGm1Wo5xdbH6HEAejZfCqA
</commit_message>
<xml_diff>
--- a/cantidades/Cantidades_Multifamiliar_Herrera.xlsx
+++ b/cantidades/Cantidades_Multifamiliar_Herrera.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="727" uniqueCount="489">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="727" uniqueCount="488">
   <si>
     <t xml:space="preserve">RESUMEN DE CANTIDADES PRINCIPALES — MULTIFAMILIAR HERRERA</t>
   </si>
@@ -1329,7 +1329,7 @@
     <t xml:space="preserve">Columnas 40×40 — longitudinal</t>
   </si>
   <si>
-    <t xml:space="preserve">Confirmado: 4 #4 por columna (L=1.85 del detalle)</t>
+    <t xml:space="preserve">Confirmado: 4 #4 por columna, L=1.80</t>
   </si>
   <si>
     <t xml:space="preserve">Columnas 40×40 — flejes cerrados</t>
@@ -1437,16 +1437,13 @@
     <t xml:space="preserve">Resuelto</t>
   </si>
   <si>
-    <t xml:space="preserve">Columnas 40×40: confirmado 4 #4 por columna (16 barras en total). Se tomó L=1.85 m del detalle de refuerzo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirmado por el arquitecto. Verificar que la longitud de 1.85 m quede en la cartilla final.</t>
+    <t xml:space="preserve">Columnas 40×40: confirmado 4 #4 por columna (16 barras en total). Longitud total confirmada L=1.80 m.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmado por el arquitecto.</t>
   </si>
   <si>
     <t xml:space="preserve">Flejes: confirmado fleje #3 @0.075 con L=1.48 m (80 flejes en total).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirmado por el arquitecto.</t>
   </si>
   <si>
     <t xml:space="preserve">EST-02</t>
@@ -2330,7 +2327,7 @@
       </c>
       <c r="B13" s="6" t="n">
         <f aca="false">('Foso ascensor'!K53+'Foso ascensor'!K54)*(1+Supuestos!$B$6)</f>
-        <v>342.85986</v>
+        <v>342.0249</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>25</v>
@@ -2722,7 +2719,7 @@
       <c r="I14" s="5"/>
       <c r="J14" s="10" t="n">
         <f aca="false">'Foso ascensor'!K53*(1+Supuestos!$B$6)</f>
-        <v>273.24066</v>
+        <v>272.4057</v>
       </c>
       <c r="K14" s="11" t="s">
         <v>58</v>
@@ -7562,11 +7559,11 @@
         <v>16</v>
       </c>
       <c r="H51" s="29" t="n">
-        <v>1.85</v>
+        <v>1.8</v>
       </c>
       <c r="I51" s="18" t="n">
         <f aca="false">G51*H51</f>
-        <v>29.6</v>
+        <v>28.8</v>
       </c>
       <c r="J51" s="38" t="n">
         <f aca="false">Supuestos!$B$5</f>
@@ -7574,7 +7571,7 @@
       </c>
       <c r="K51" s="18" t="n">
         <f aca="false">I51*J51</f>
-        <v>29.4224</v>
+        <v>28.6272</v>
       </c>
       <c r="L51" s="5" t="s">
         <v>433</v>
@@ -7637,12 +7634,12 @@
       <c r="H53" s="2"/>
       <c r="I53" s="36" t="n">
         <f aca="false">SUMIF(B45:B52,"#4",I45:I52)</f>
-        <v>261.8</v>
+        <v>261</v>
       </c>
       <c r="J53" s="2"/>
       <c r="K53" s="36" t="n">
         <f aca="false">SUMIF(B45:B52,"#4",K45:K52)</f>
-        <v>260.2292</v>
+        <v>259.434</v>
       </c>
       <c r="L53" s="2"/>
     </row>
@@ -7683,7 +7680,7 @@
       <c r="J55" s="2"/>
       <c r="K55" s="40" t="n">
         <f aca="false">(K53+K54)/B29</f>
-        <v>120.137306843267</v>
+        <v>119.844738778514</v>
       </c>
       <c r="L55" s="2"/>
     </row>
@@ -8002,7 +7999,7 @@
         <v>471</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8010,13 +8007,13 @@
         <v>8</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>473</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="D11" s="5" t="s">
         <v>474</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>475</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8024,13 +8021,13 @@
         <v>9</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="C12" s="5" t="s">
+        <v>475</v>
+      </c>
+      <c r="D12" s="5" t="s">
         <v>476</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>477</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8038,13 +8035,13 @@
         <v>10</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="C13" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>478</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>479</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8052,13 +8049,13 @@
         <v>11</v>
       </c>
       <c r="B14" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>480</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>481</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8066,13 +8063,13 @@
         <v>12</v>
       </c>
       <c r="B15" s="5" t="s">
+        <v>482</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>483</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="5" t="s">
         <v>484</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>485</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8080,13 +8077,13 @@
         <v>13</v>
       </c>
       <c r="B16" s="5" t="s">
+        <v>485</v>
+      </c>
+      <c r="C16" s="5" t="s">
         <v>486</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="D16" s="5" t="s">
         <v>487</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>488</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Foso: formas reales de las barras (ganchos a 180° y patas a 90°)
Corrige el figurado de los verticales de muro, el longitudinal de
columnas y las barras de losa según los cortes y el detalle del EST-02.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGm1Wo5xdbH6HEAejZfCqA
</commit_message>
<xml_diff>
--- a/cantidades/Cantidades_Multifamiliar_Herrera.xlsx
+++ b/cantidades/Cantidades_Multifamiliar_Herrera.xlsx
@@ -1296,40 +1296,40 @@
     <t xml:space="preserve">#4</t>
   </si>
   <si>
-    <t xml:space="preserve">Corte A-A: #4 c/0.20 L=2.20 (doble parrilla)</t>
+    <t xml:space="preserve">Corte A-A: recto 1.70 + gancho 180° de 0.20 en cada extremo, L=2.20 (doble parrilla)</t>
   </si>
   <si>
     <t xml:space="preserve">Losa fondo — barras sentido Y (largo)</t>
   </si>
   <si>
-    <t xml:space="preserve">Corte B-B: #4 c/0.20 L=2.60 (doble parrilla)</t>
+    <t xml:space="preserve">Corte B-B: recto 2.10 + gancho 180° de 0.20 en cada extremo, L=2.60 (doble parrilla)</t>
   </si>
   <si>
     <t xml:space="preserve">Muros sentido X — horizontales</t>
   </si>
   <si>
-    <t xml:space="preserve">Planta refuerzo: #4 c/0.20 L=2.10</t>
+    <t xml:space="preserve">Planta refuerzo: recto 1.68 + patas a 90° de 0.20, L=2.10</t>
   </si>
   <si>
     <t xml:space="preserve">Muros sentido Y — horizontales</t>
   </si>
   <si>
-    <t xml:space="preserve">Planta refuerzo: #4 c/0.20 L=2.50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Muros sentido X — verticales (gancho a losa)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cortes A-A/B-B: #4 c/0.20 L=1.75</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Muros sentido Y — verticales (gancho a losa)</t>
+    <t xml:space="preserve">Planta refuerzo: recto 2.08 + patas a 90° de 0.20, L=2.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muros sentido X — verticales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cortes: recto 1.28 + gancho sup. 180° de 0.20 + pata inf. 90° de 0.20, L=1.75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muros sentido Y — verticales</t>
   </si>
   <si>
     <t xml:space="preserve">Columnas 40×40 — longitudinal</t>
   </si>
   <si>
-    <t xml:space="preserve">Confirmado: 4 #4 por columna, L=1.80</t>
+    <t xml:space="preserve">Confirmado: 4 #4 por columna, recto 1.32 + gancho sup. 180° de 0.20 + pata inf. 90° de 0.20, L=1.80</t>
   </si>
   <si>
     <t xml:space="preserve">Columnas 40×40 — flejes cerrados</t>
@@ -1446,13 +1446,13 @@
     <t xml:space="preserve">Flejes: confirmado fleje #3 @0.075 con L=1.48 m (80 flejes en total).</t>
   </si>
   <si>
+    <t xml:space="preserve">Longitudes: L=2.20/2.60 son las barras de losa (ganchos a 180°) y L=2.10/2.50 las horizontales de muro (patas a 90°). Son barras distintas, no hay inconsistencia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ninguna.</t>
+  </si>
+  <si>
     <t xml:space="preserve">EST-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Barras de losa: la planta indica L=2.10/2.50 y los cortes L=2.20/2.60. Se usaron las de los cortes (losa) y las de planta (horizontales de muros).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirmar la cartilla de hierros con el calculista.</t>
   </si>
   <si>
     <t xml:space="preserve">La lámina no indica f'c del concreto, fy del acero, recubrimientos generales ni tipo exacto de perfil (HEA/HEB 200). Se asumió 21 MPa, 420 MPa y HEB 200.</t>
@@ -7277,7 +7277,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
         <v>420</v>
       </c>
@@ -7320,7 +7320,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
         <v>423</v>
       </c>
@@ -7363,7 +7363,7 @@
         <v>424</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
         <v>425</v>
       </c>
@@ -7407,7 +7407,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
         <v>427</v>
       </c>
@@ -7451,7 +7451,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
         <v>429</v>
       </c>
@@ -7495,7 +7495,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
         <v>431</v>
       </c>
@@ -7539,7 +7539,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
         <v>432</v>
       </c>
@@ -8007,13 +8007,13 @@
         <v>8</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>468</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>472</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="D11" s="5" t="s">
         <v>473</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>474</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8021,7 +8021,7 @@
         <v>9</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>475</v>
@@ -8035,7 +8035,7 @@
         <v>10</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>477</v>

</xml_diff>

<commit_message>
Foso: fleje de columnas L=1.50 m; PDF y Excel de cartilla de acero y concreto por elementos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGm1Wo5xdbH6HEAejZfCqA
</commit_message>
<xml_diff>
--- a/cantidades/Cantidades_Multifamiliar_Herrera.xlsx
+++ b/cantidades/Cantidades_Multifamiliar_Herrera.xlsx
@@ -270,7 +270,7 @@
     <t xml:space="preserve">Acero de refuerzo #3 (3/8") — flejes</t>
   </si>
   <si>
-    <t xml:space="preserve">Acero corrugado fy = 420 MPa, NTC 2289. Flejes cerrados #3 @0.075 m, L = 1.48 m, gancho a 135°.</t>
+    <t xml:space="preserve">Acero corrugado fy = 420 MPa, NTC 2289. Flejes cerrados #3 @0.075 m, L = 1.50 m, gancho a 135°.</t>
   </si>
   <si>
     <t xml:space="preserve">2.8</t>
@@ -1338,7 +1338,7 @@
     <t xml:space="preserve">#3</t>
   </si>
   <si>
-    <t xml:space="preserve">Confirmado: fleje #3 @0.075 L=1.48</t>
+    <t xml:space="preserve">Confirmado: fleje #3 @0.075 L=1.50</t>
   </si>
   <si>
     <t xml:space="preserve">Subtotal #4 (sin desperdicio)</t>
@@ -1443,7 +1443,7 @@
     <t xml:space="preserve">Confirmado por el arquitecto.</t>
   </si>
   <si>
-    <t xml:space="preserve">Flejes: confirmado fleje #3 @0.075 con L=1.48 m (80 flejes en total).</t>
+    <t xml:space="preserve">Flejes: confirmado fleje #3 @0.075 con L=1.50 m (80 flejes en total).</t>
   </si>
   <si>
     <t xml:space="preserve">Longitudes: L=2.20/2.60 son las barras de losa (ganchos a 180°) y L=2.10/2.50 las horizontales de muro (patas a 90°). Son barras distintas, no hay inconsistencia.</t>
@@ -2327,7 +2327,7 @@
       </c>
       <c r="B13" s="6" t="n">
         <f aca="false">('Foso ascensor'!K53+'Foso ascensor'!K54)*(1+Supuestos!$B$6)</f>
-        <v>342.0249</v>
+        <v>342.9657</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>25</v>
@@ -2748,7 +2748,7 @@
       <c r="I15" s="5"/>
       <c r="J15" s="10" t="n">
         <f aca="false">'Foso ascensor'!K54*(1+Supuestos!$B$6)</f>
-        <v>69.6192</v>
+        <v>70.56</v>
       </c>
       <c r="K15" s="11" t="s">
         <v>58</v>
@@ -7603,11 +7603,11 @@
         <v>80</v>
       </c>
       <c r="H52" s="29" t="n">
-        <v>1.48</v>
+        <v>1.5</v>
       </c>
       <c r="I52" s="18" t="n">
         <f aca="false">G52*H52</f>
-        <v>118.4</v>
+        <v>120</v>
       </c>
       <c r="J52" s="38" t="n">
         <f aca="false">Supuestos!$B$4</f>
@@ -7615,7 +7615,7 @@
       </c>
       <c r="K52" s="18" t="n">
         <f aca="false">I52*J52</f>
-        <v>66.304</v>
+        <v>67.2</v>
       </c>
       <c r="L52" s="5" t="s">
         <v>436</v>
@@ -7656,12 +7656,12 @@
       <c r="H54" s="2"/>
       <c r="I54" s="36" t="n">
         <f aca="false">SUMIF(B45:B52,"#3",I45:I52)</f>
-        <v>118.4</v>
+        <v>120</v>
       </c>
       <c r="J54" s="2"/>
       <c r="K54" s="36" t="n">
         <f aca="false">SUMIF(B45:B52,"#3",K45:K52)</f>
-        <v>66.304</v>
+        <v>67.2</v>
       </c>
       <c r="L54" s="2"/>
     </row>
@@ -7680,7 +7680,7 @@
       <c r="J55" s="2"/>
       <c r="K55" s="40" t="n">
         <f aca="false">(K53+K54)/B29</f>
-        <v>119.844738778514</v>
+        <v>120.174392935982</v>
       </c>
       <c r="L55" s="2"/>
     </row>

</xml_diff>

<commit_message>
Foso: acero en metros lineales en lugar de kg
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGm1Wo5xdbH6HEAejZfCqA
</commit_message>
<xml_diff>
--- a/cantidades/Cantidades_Multifamiliar_Herrera.xlsx
+++ b/cantidades/Cantidades_Multifamiliar_Herrera.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="727" uniqueCount="488">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="727" uniqueCount="489">
   <si>
     <t xml:space="preserve">RESUMEN DE CANTIDADES PRINCIPALES — MULTIFAMILIAR HERRERA</t>
   </si>
@@ -105,1264 +105,1267 @@
     <t xml:space="preserve">Foso ascensor — acero de refuerzo total (con desperdicio)</t>
   </si>
   <si>
+    <t xml:space="preserve">ml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#4 + #3, metros lineales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Foso ascensor — excavación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CUADRO DE CANTIDADES DE OBRA — MULTIFAMILIAR HERRERA (Puerto Berrío, Antioquia)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alcance: niveles P1–P5 terminados en el modelo Revit + foso de ascensor (plano EST-02). Sin precios: el presupuesto se maneja aparte. Fuente: R = medido en Revit · E = plano estructural EST-02 · D = derivada por fórmula (ver hoja Supuestos) · P = por confirmar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ítem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Descripción</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Especificación técnica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cantidad total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Observaciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRELIMINARES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Localización, trazado y replanteo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Con equipo de topografía (estación total / nivel). Incluye referencias de ejes y niveles, mojones y estacas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R/D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Área cubierta total P1–P5 + área exterior P1 (área de intervención por nivel).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Localización y replanteo del foso de ascensor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replanteo de ejes A-B / 1-2 según planta de geometría EST-02 (cotas a ejes: 1.10, 1.25, 1.19, 1.34 m).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Huella 2.10 × 2.50 m.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FOSO DE ASCENSOR — CIMENTACIÓN Y ESTRUCTURA (EST-02)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excavación manual en material común</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hasta cota N-1.55 (fondo de solado), con sobreancho de 0.30 m por lado. Incluye perfilado de fondo. Precaución: zapatas vecinas en ejes A y B (NSZ-2.00 / NIZ-2.50) — no descalzar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E/D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solado de limpieza e=0.05 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concreto pobre f'c = 14 MPa (2.000 psi) bajo losa de fondo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No dibujado en EST-02; recomendado. Incluye desperdicio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concreto losa de fondo e=0.20 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concreto f'c = 21 MPa (3.000 psi) con aditivo impermeabilizante integral. Cara superior a N-1.30, inferior N-1.50. Recubrimiento 75 mm contra suelo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incluye desperdicio. f'c NO indicado en EST-02: confirmar en notas generales (EST-01).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concreto muros de contención e=0.15 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concreto f'c = 21 MPa (3.000 psi) con aditivo impermeabilizante integral, h = 1.20 m sobre losa (hasta N-0.10).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incluye desperdicio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concreto columnas 40×40 cm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concreto f'c = 21 MPa (3.000 psi). 4 und, de N-1.50 a N-0.10 (h = 1.40 m). Reciben perfil HE 200.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acero de refuerzo #4 (1/2")</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acero corrugado fy = 420 MPa (60.000 psi), NTC 2289. Losa doble parrilla #4 c/0.20; muros #4 c/0.20 en ambos sentidos; longitudinal de columnas 4 #4 por columna. Figurado según cartilla (hoja Foso ascensor).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metros lineales de barra. Incluye desperdicio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acero de refuerzo #3 (3/8") — flejes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acero corrugado fy = 420 MPa, NTC 2289. Flejes cerrados #3 @0.075 m, L = 1.50 m, gancho a 135°.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formaleta para muros y columnas del foso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formaleta metálica o en madera cepillada, con desmoldante. Ambas caras de muros + caras exteriores de columnas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Impermeabilización interior del foso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mortero impermeable cementicio (2 manos cruzadas) en fondo y muros + mediacaña en encuentros muro-losa. Rematar a N-0.10.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No especificado en EST-02. Recomendado (foso bajo nivel de terreno).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relleno compactado perimetral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Material seleccionado de excavación o recebo, en capas ≤ 0.20 m compactadas al 95 % Proctor modificado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retiro de sobrantes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cargue, transporte y disposición en sitio autorizado (escombrera).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Volumen suelto (con expansión).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Platina base A36 300×300×16 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acero ASTM A36, 4 perforaciones para pernos Ø5/8". Nivelada con mortero sin retracción (grouting).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peso total en hoja Foso ascensor.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pernos de anclaje Ø5/8" con gancho</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barra roscada ASTM F1554 Gr. 36 (o A307), embebido 314 mm, tuerca y arandela. 4 por platina.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Soldadura de filete 5/16"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Electrodo E70XX, todo el contorno del perfil HE 200 a la platina.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Longitud aproximada por contorno de perfil.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perfil HE 200 — columnas metálicas del ducto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perfil HE 200 (se asume HEB 200 = 61.3 kg/m), ASTM A572 Gr. 50 o A36, con anticorrosivo + esmalte.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E/P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cantidad en ml PENDIENTE: depende de la altura total del ducto (no está en EST-02).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MAMPOSTERÍA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muro en mampostería de arcilla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unidad de arcilla cocida NTC 4205 (tipo y espesor a confirmar), pega con mortero 1:4 tipo S (NTC 3329), juntas de 1 cm. Área neta medida en Revit (descuenta vanos, sin guardaescoba).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">131 muros en P1–P5.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unidades de mampostería (referencia)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bloque de arcilla 10×20×30 cm (supuesto). Incluye desperdicio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ajustar rendimiento en Supuestos según la unidad especificada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mortero de pega 1:4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cemento gris + arena de pega, f'cm ≥ 12.5 MPa (tipo S).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PAÑETES Y ACABADOS DE MUROS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pañete liso sobre muros (ambas caras)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mortero 1:4, e = 1.5 cm promedio, a plomo y regla. En fachada usar mortero 1:3 con impermeabilizante integral.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bruto: descontar las zonas que lleven enchape (baños, cocinas) cuando se definan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estuco + pintura vinilo tipo 1 (3 manos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estuco plástico + vinilo tipo 1 NTC 1335, color a definir. Fachada: pintura para exteriores (elastomérica o acrílica).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Misma área bruta que el pañete; descontar enchapes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dinteles sobre vanos (puertas y ventanas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dintel en concreto 21 MPa o en perfil, apoyo 0.20 m por lado. Ancho del muro.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No incluye puertas de vestier Häfele (sin medida en el modelo).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PISOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alistado de piso (mortero de nivelación)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mortero 1:4, e = 4 cm, nivelado y afinado para recibir acabado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Área cubierta por nivel (Revit).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mortero para alistado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mortero 1:4.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acabado de piso interior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo POR DEFINIR (porcelanato / cerámica antideslizante en baños y balcones). Incluye pegante y boquilla.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R/P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Área bruta; descontar muros si el área de Revit los incluye. Guardaescoba pendiente (perímetro de rooms).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Piso exterior / andén P1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concreto 21 MPa e = 8 cm sobre recebo compactado, o adoquín. Acabado antideslizante.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CIELORRASOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cielorraso interior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo POR DEFINIR: pañete bajo placa + estuco y vinilo, o drywall en placa de yeso 1/2". En baños usar placa RH.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D/P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aproximado = área cubierta por nivel. Confirmar con plano de cielos (RCP).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CARPINTERÍA — PUERTAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta de garaje — 2.4 × 2.1 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta metálica enrollable o seccional, lámina cal. 20, con cerradura de seguridad.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta principal de acceso — 0.9 × 2.1 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta de seguridad metálica o en madera maciza, marco metálico cal. 18, cerradura de seguridad y mirilla.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta de acceso secundario — 0.915 × 2.13 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta corrediza social (balcón) — 1.2 × 2.1 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta corrediza en aluminio con vidrio de seguridad templado 6 mm (NSR-10 Título K).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta corrediza de habitación/closet — 0.9 × 2.1 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hoja corrediza entamborada en MDF, herraje de riel superior, manija embutida.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta corrediza de baño/closet menor — 0.7 × 2.1 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta batiente de habitación — 0.8 × 2.1 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hoja entamborada en MDF, marco en madera, bisagras de 3½" y cerradura de pomo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta batiente de habitación — 0.9 × 2.1 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta batiente de baño/closet — 0.7 × 2.1 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hoja entamborada en MDF RH (resistente a humedad), marco en madera, cerradura de baño.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta principal de apartamento — 1 × 2.1 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta-ventanal corrediza (balcón) — 1.6 × 2.3 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta corrediza de vestier (herraje Häfele) — ≈7.73 m² de hoja (total Revit)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puertas corredizas de vestier con herraje Häfele, hoja en MDF/aglomerado enchapado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VENTANERÍA Y VIDRIOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ventana de habitación — 0.8 × 0.8 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ventana en aluminio (proyectante o corrediza), vidrio incoloro 4 mm, empaques y sellos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ventana de baño/cocina — 0.91 × 0.91 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ventana en aluminio, vidrio esmerilado/sandblasting 4 mm (privacidad), con celosía de ventilación.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ventanal de circulación (hall/escalera) — 0.9 × 2.41 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perfilería en aluminio, vidrio de seguridad laminado o templado 6 mm (vano a piso, NSR-10 Título K).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ventanal de fachada — acceso — 0.68 × 2.2 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Área de vidrio en ventanas y ventanales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suma de ancho × alto × cantidad.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No incluye vidrio de puertas-ventanal (ver ítem siguiente).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Área de vidrio de seguridad en puertas-ventanal y puerta de balcón</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vidrio templado 6 mm.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alfajías en ventanas (excepto vanos a piso)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alfajía prefabricada en concreto o granito, con gotero, pendiente hacia el exterior.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solo ventanas de habitación y baño/cocina.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">APARATOS SANITARIOS, GRIFERÍAS E INCRUSTACIONES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sanitario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sanitario de porcelana vitrificada, tanque de bajo consumo (≤ 4.8 L/descarga, NTC 920), con grifería de llenado y asiento.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cabina de ducha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zona de ducha con piso en cerámica antideslizante, pendiente 1–2 % al sifón; cabina según modelo Revit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regadera de ducha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regadera + mezclador monocontrol cromado (agua fría/caliente), sistema ahorrador.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ducha accesible (con barras)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ducha a nivel sin sardinel, asiento abatible y barras de apoyo en acero inoxidable (NTC 6047 accesibilidad).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lavamanos de baño</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lavamanos de porcelana (de incrustar u ovalín), con sifón, desagüe y grifería monocontrol ahorradora.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mampara de baño</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mampara en vidrio templado 8 mm con perfilería en aluminio (NSR-10 Título K).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grifería de lavamanos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monocontrol cromada, aireador ahorrador.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 por lavamanos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mezclador de ducha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monocontrol empotrado, cartucho cerámico.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regaderas + ducha accesible.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Juego de incrustaciones por baño</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toallero, jabonera, portarrollos y gancho, en porcelana o acero inoxidable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 juego por baño (= N° de sanitarios).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sifón de piso 3" con rejilla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PVC sanitario + rejilla en acero inoxidable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mínimo 1 por ducha; agregar los de cocina/zona de ropas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EQUIPO DE ASCENSOR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ascensor de pasajeros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ascensor eléctrico sin cuarto de máquinas (MRL), capacidad y paradas POR DEFINIR (6 niveles), NTC 5926 / EN 81-20. Incluye cabina, puertas de piso, guías, contrapeso y control.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QA crítico: el ascensor no está modelado en Revit. El foso de EST-02 tiene luz libre 1.50 × 1.90 m: validar con el proveedor.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUPUESTOS Y PARÁMETROS DE CÁLCULO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Celdas en azul con fondo amarillo = parámetros editables. Al cambiarlos se recalculan todas las cantidades derivadas. Fuente indicada en la columna D.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parámetro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuente / criterio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peso nominal barra #3 (3/8")</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kg/m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NSR-10 / NTC 2289</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peso nominal barra #4 (1/2")</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desperdicio acero de refuerzo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Criterio usual de obra (traslapos y cortes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desperdicio concreto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Criterio usual de obra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unidades de mampostería por m² (bloque arcilla 10×20×30 cm, junta 1 cm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">un/m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1/(0.31×0.21). AJUSTAR si la unidad especificada es otra (p.ej. tolete 6×12×24 ≈ 54 un/m² en soga)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desperdicio unidades de mampostería</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mortero de pega por m² de muro (bloque e=10 cm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m³/m²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rendimiento de referencia; ajustar según unidad y espesor de junta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Caras de pañete/estuco/pintura por muro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">caras</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supuesto: todos los muros se revocan por ambas caras (bruto, sin descontar enchapes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Espesor de alistado (mortero de nivelación) de piso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supuesto de diseño; confirmar con nivel de acabado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sobreancho de excavación por lado (foso)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Espacio de trabajo para formaleta exterior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profundidad de excavación foso (desde N-0.10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N-0.10 a N-1.50 (EST-02) + 0.05 de solado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Factor de expansión del suelo (sobrantes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Criterio usual para material común</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Espesor solado de limpieza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recomendado bajo losa en contacto con suelo (no dibujado en EST-02)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sobreancho solado por lado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Criterio usual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Densidad acero estructural</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kg/m³</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor estándar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peso perfil HE 200 (se asume HEB 200)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HEB 200 = 61.3 kg/m; si es HEA 200 usar 42.3 kg/m. EST-02 no lo precisa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apoyo de dintel por lado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Criterio usual en mampostería</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recubrimiento de impermeabilización interior foso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 = incluir (recomendado para foso bajo nivel de piso)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DATOS DE ENTRADA — EXTRAÍDOS DEL MODELO REVIT (MULTIF H - RVT.rvt)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuente: dashboard index.html (consulta directa al modelo). Solo niveles P1–P5 terminados; P6/P7 y cubierta en diseño, NO incluidos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. SUPERFICIES Y MUROS POR NIVEL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concepto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Área cubierta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Programa de superficies Revit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Área exterior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solo P1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N° de muros de mampostería</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Área de muros de mampostería (neta, una cara)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revit descuenta vanos de puertas/ventanas. Sin guardaescoba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. PUERTAS — por función y medida</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Función</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ancho (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alto (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta de garaje</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta principal de acceso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta de acceso secundario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medida imperial 3'×7'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta corrediza social (balcón)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta corrediza de habitación/closet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta corrediza de baño/closet menor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta batiente de habitación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta batiente de baño/closet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta principal de apartamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta-ventanal corrediza (balcón)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Puerta corrediza de vestier (herraje Häfele)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revit reporta ≈7.73 m² de hoja; sin ancho/alto definido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL PUERTAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. VENTANAS Y VENTANALES — por función y medida</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ventana de habitación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ventana de baño/cocina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ventanal de circulación (hall/escalera)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panel de muro cortina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ventanal de fachada — acceso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL VENTANAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. APARATOS SANITARIOS — verificados elemento por elemento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aparato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL APARATOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MEMORIA DE CÁLCULO — FOSO DE ASCENSOR (plano EST-02, versión 01, 19/06/2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diseño estructural: A3 Ingeniería. Escala 1:25. Cotas en m. Valores en azul tomados del plano; las cantidades son fórmulas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A. GEOMETRÍA (según planta, cortes A-A y B-B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dato</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luz libre interior del foso — sentido X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planta foso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luz libre interior del foso — sentido Y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Espesor muros de concreto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planta foso: Muro e=0.15m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lado columna cuadrada (4 und, en esquinas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Columna 40×40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Número de columnas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distancia libre entre caras de columnas — X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distancia libre entre caras de columnas — Y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Altura total foso (N-0.10 a N-1.50)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cortes A-A / B-B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Espesor losa de fondo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Losa e=0.20m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Losa — dimensión exterior X (luz + 2 muros)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Losa — dimensión exterior Y (luz + 2 muros)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Huella total con columnas — X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Huella total con columnas — Y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Traslapo columna–losa por esquina (lado)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Altura libre muros (sobre losa)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profundidad útil del foso (N-0.10 a cara superior losa)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verificar contra la ficha técnica del ascensor elegido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B. CONCRETO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elemento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cant.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cálculo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Columnas 40×40 (altura total foso)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 × 0.40 × 0.40 × 1.40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Losa de fondo e=0.20 (descontando columnas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.80 × 2.20 × 0.20 − 4 × 0.25² × 0.20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muros e=0.15 (entre columnas, sobre losa)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(2×1.30 + 2×1.70) × 1.20 × 0.15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solado de limpieza (concreto pobre)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(1.80+0.20) × (2.20+0.20) × 0.05 — recomendado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL CONCRETO ESTRUCTURAL (sin desperdicio)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C. MOVIMIENTO DE TIERRA Y FORMALETA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excavación manual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(2.10+0.60) × (2.50+0.60) × 1.45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Volumen ocupado por el foso + solado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Huella real (losa + salientes de columnas) × 1.40 + solado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relleno compactado perimetral (material seleccionado)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excavación − volumen ocupado. Compactar en capas ≤ 0.20 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Retiro de sobrantes (suelto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(Excavación − relleno) × factor de expansión</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formaleta muros — cara interior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perímetro interior 6.80 × 1.20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formaleta muros — cara exterior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tramos entre columnas 6.00 × 1.40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formaleta columnas — caras exteriores expuestas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 × (2×0.40 + 2×0.15) × 1.40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL FORMALETA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Impermeabilización interior (fondo + muros)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.50×1.90 + 6.80×1.20 — no especificado en EST-02, recomendado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D. CARTILLA DE DESPIECE — ACERO DE REFUERZO fy = 420 MPa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Elemento / posición</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Barra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Separación (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Long. a distribuir (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N° barras por capa/elem.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capas o elementos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N° barras total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L barra (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Long. total (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peso (kg)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fuente en plano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Losa fondo — barras sentido X (corto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corte A-A: recto 1.70 + gancho 180° de 0.20 en cada extremo, L=2.20 (doble parrilla)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Losa fondo — barras sentido Y (largo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corte B-B: recto 2.10 + gancho 180° de 0.20 en cada extremo, L=2.60 (doble parrilla)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muros sentido X — horizontales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planta refuerzo: recto 1.68 + patas a 90° de 0.20, L=2.10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muros sentido Y — horizontales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planta refuerzo: recto 2.08 + patas a 90° de 0.20, L=2.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muros sentido X — verticales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cortes: recto 1.28 + gancho sup. 180° de 0.20 + pata inf. 90° de 0.20, L=1.75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muros sentido Y — verticales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Columnas 40×40 — longitudinal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmado: 4 #4 por columna, recto 1.32 + gancho sup. 180° de 0.20 + pata inf. 90° de 0.20, L=1.80</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Columnas 40×40 — flejes cerrados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirmado: fleje #3 @0.075 L=1.50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtotal #4 (sin desperdicio)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtotal #3 (sin desperdicio)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cuantía de referencia (kg acero / m³ concreto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E. ESTRUCTURA METÁLICA — DETALLE CONEXIÓN 1 (perfil HE 200 a columna 40×40)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Especificación / cálculo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Platina base A36 300×300×16 mm — unidades</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 por columna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Platina base A36 300×300×16 mm — peso</t>
+  </si>
+  <si>
     <t xml:space="preserve">kg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#4 + #3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Foso ascensor — excavación</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CUADRO DE CANTIDADES DE OBRA — MULTIFAMILIAR HERRERA (Puerto Berrío, Antioquia)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alcance: niveles P1–P5 terminados en el modelo Revit + foso de ascensor (plano EST-02). Sin precios: el presupuesto se maneja aparte. Fuente: R = medido en Revit · E = plano estructural EST-02 · D = derivada por fórmula (ver hoja Supuestos) · P = por confirmar.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ítem</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Descripción</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Especificación técnica</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cantidad total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Observaciones</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PRELIMINARES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Localización, trazado y replanteo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Con equipo de topografía (estación total / nivel). Incluye referencias de ejes y niveles, mojones y estacas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R/D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Área cubierta total P1–P5 + área exterior P1 (área de intervención por nivel).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Localización y replanteo del foso de ascensor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replanteo de ejes A-B / 1-2 según planta de geometría EST-02 (cotas a ejes: 1.10, 1.25, 1.19, 1.34 m).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Huella 2.10 × 2.50 m.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FOSO DE ASCENSOR — CIMENTACIÓN Y ESTRUCTURA (EST-02)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Excavación manual en material común</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hasta cota N-1.55 (fondo de solado), con sobreancho de 0.30 m por lado. Incluye perfilado de fondo. Precaución: zapatas vecinas en ejes A y B (NSZ-2.00 / NIZ-2.50) — no descalzar.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E/D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solado de limpieza e=0.05 m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Concreto pobre f'c = 14 MPa (2.000 psi) bajo losa de fondo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No dibujado en EST-02; recomendado. Incluye desperdicio.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Concreto losa de fondo e=0.20 m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Concreto f'c = 21 MPa (3.000 psi) con aditivo impermeabilizante integral. Cara superior a N-1.30, inferior N-1.50. Recubrimiento 75 mm contra suelo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Incluye desperdicio. f'c NO indicado en EST-02: confirmar en notas generales (EST-01).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Concreto muros de contención e=0.15 m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Concreto f'c = 21 MPa (3.000 psi) con aditivo impermeabilizante integral, h = 1.20 m sobre losa (hasta N-0.10).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Incluye desperdicio.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Concreto columnas 40×40 cm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Concreto f'c = 21 MPa (3.000 psi). 4 und, de N-1.50 a N-0.10 (h = 1.40 m). Reciben perfil HE 200.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acero de refuerzo #4 (1/2")</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acero corrugado fy = 420 MPa (60.000 psi), NTC 2289. Losa doble parrilla #4 c/0.20; muros #4 c/0.20 en ambos sentidos; longitudinal de columnas 4 #4 por columna. Figurado según cartilla (hoja Foso ascensor).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acero de refuerzo #3 (3/8") — flejes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acero corrugado fy = 420 MPa, NTC 2289. Flejes cerrados #3 @0.075 m, L = 1.50 m, gancho a 135°.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Formaleta para muros y columnas del foso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Formaleta metálica o en madera cepillada, con desmoldante. Ambas caras de muros + caras exteriores de columnas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Impermeabilización interior del foso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mortero impermeable cementicio (2 manos cruzadas) en fondo y muros + mediacaña en encuentros muro-losa. Rematar a N-0.10.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No especificado en EST-02. Recomendado (foso bajo nivel de terreno).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Relleno compactado perimetral</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Material seleccionado de excavación o recebo, en capas ≤ 0.20 m compactadas al 95 % Proctor modificado.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Retiro de sobrantes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cargue, transporte y disposición en sitio autorizado (escombrera).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Volumen suelto (con expansión).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Platina base A36 300×300×16 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acero ASTM A36, 4 perforaciones para pernos Ø5/8". Nivelada con mortero sin retracción (grouting).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peso total en hoja Foso ascensor.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pernos de anclaje Ø5/8" con gancho</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Barra roscada ASTM F1554 Gr. 36 (o A307), embebido 314 mm, tuerca y arandela. 4 por platina.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Soldadura de filete 5/16"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Electrodo E70XX, todo el contorno del perfil HE 200 a la platina.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ml</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Longitud aproximada por contorno de perfil.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Perfil HE 200 — columnas metálicas del ducto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Perfil HE 200 (se asume HEB 200 = 61.3 kg/m), ASTM A572 Gr. 50 o A36, con anticorrosivo + esmalte.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E/P</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cantidad en ml PENDIENTE: depende de la altura total del ducto (no está en EST-02).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MAMPOSTERÍA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Muro en mampostería de arcilla</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unidad de arcilla cocida NTC 4205 (tipo y espesor a confirmar), pega con mortero 1:4 tipo S (NTC 3329), juntas de 1 cm. Área neta medida en Revit (descuenta vanos, sin guardaescoba).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">131 muros en P1–P5.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unidades de mampostería (referencia)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bloque de arcilla 10×20×30 cm (supuesto). Incluye desperdicio.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ajustar rendimiento en Supuestos según la unidad especificada.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mortero de pega 1:4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cemento gris + arena de pega, f'cm ≥ 12.5 MPa (tipo S).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PAÑETES Y ACABADOS DE MUROS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pañete liso sobre muros (ambas caras)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mortero 1:4, e = 1.5 cm promedio, a plomo y regla. En fachada usar mortero 1:3 con impermeabilizante integral.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bruto: descontar las zonas que lleven enchape (baños, cocinas) cuando se definan.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estuco + pintura vinilo tipo 1 (3 manos)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estuco plástico + vinilo tipo 1 NTC 1335, color a definir. Fachada: pintura para exteriores (elastomérica o acrílica).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Misma área bruta que el pañete; descontar enchapes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dinteles sobre vanos (puertas y ventanas)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dintel en concreto 21 MPa o en perfil, apoyo 0.20 m por lado. Ancho del muro.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No incluye puertas de vestier Häfele (sin medida en el modelo).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PISOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alistado de piso (mortero de nivelación)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mortero 1:4, e = 4 cm, nivelado y afinado para recibir acabado.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Área cubierta por nivel (Revit).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mortero para alistado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mortero 1:4.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acabado de piso interior</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tipo POR DEFINIR (porcelanato / cerámica antideslizante en baños y balcones). Incluye pegante y boquilla.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R/P</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Área bruta; descontar muros si el área de Revit los incluye. Guardaescoba pendiente (perímetro de rooms).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Piso exterior / andén P1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Concreto 21 MPa e = 8 cm sobre recebo compactado, o adoquín. Acabado antideslizante.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CIELORRASOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cielorraso interior</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tipo POR DEFINIR: pañete bajo placa + estuco y vinilo, o drywall en placa de yeso 1/2". En baños usar placa RH.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D/P</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aproximado = área cubierta por nivel. Confirmar con plano de cielos (RCP).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CARPINTERÍA — PUERTAS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta de garaje — 2.4 × 2.1 m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta metálica enrollable o seccional, lámina cal. 20, con cerradura de seguridad.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta principal de acceso — 0.9 × 2.1 m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta de seguridad metálica o en madera maciza, marco metálico cal. 18, cerradura de seguridad y mirilla.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta de acceso secundario — 0.915 × 2.13 m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta corrediza social (balcón) — 1.2 × 2.1 m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta corrediza en aluminio con vidrio de seguridad templado 6 mm (NSR-10 Título K).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta corrediza de habitación/closet — 0.9 × 2.1 m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hoja corrediza entamborada en MDF, herraje de riel superior, manija embutida.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta corrediza de baño/closet menor — 0.7 × 2.1 m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta batiente de habitación — 0.8 × 2.1 m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hoja entamborada en MDF, marco en madera, bisagras de 3½" y cerradura de pomo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta batiente de habitación — 0.9 × 2.1 m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta batiente de baño/closet — 0.7 × 2.1 m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hoja entamborada en MDF RH (resistente a humedad), marco en madera, cerradura de baño.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta principal de apartamento — 1 × 2.1 m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta-ventanal corrediza (balcón) — 1.6 × 2.3 m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta corrediza de vestier (herraje Häfele) — ≈7.73 m² de hoja (total Revit)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puertas corredizas de vestier con herraje Häfele, hoja en MDF/aglomerado enchapado.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VENTANERÍA Y VIDRIOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ventana de habitación — 0.8 × 0.8 m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ventana en aluminio (proyectante o corrediza), vidrio incoloro 4 mm, empaques y sellos.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ventana de baño/cocina — 0.91 × 0.91 m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ventana en aluminio, vidrio esmerilado/sandblasting 4 mm (privacidad), con celosía de ventilación.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ventanal de circulación (hall/escalera) — 0.9 × 2.41 m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Perfilería en aluminio, vidrio de seguridad laminado o templado 6 mm (vano a piso, NSR-10 Título K).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ventanal de fachada — acceso — 0.68 × 2.2 m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Área de vidrio en ventanas y ventanales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Suma de ancho × alto × cantidad.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No incluye vidrio de puertas-ventanal (ver ítem siguiente).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Área de vidrio de seguridad en puertas-ventanal y puerta de balcón</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vidrio templado 6 mm.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alfajías en ventanas (excepto vanos a piso)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alfajía prefabricada en concreto o granito, con gotero, pendiente hacia el exterior.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solo ventanas de habitación y baño/cocina.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">APARATOS SANITARIOS, GRIFERÍAS E INCRUSTACIONES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sanitario</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sanitario de porcelana vitrificada, tanque de bajo consumo (≤ 4.8 L/descarga, NTC 920), con grifería de llenado y asiento.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cabina de ducha</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zona de ducha con piso en cerámica antideslizante, pendiente 1–2 % al sifón; cabina según modelo Revit.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Regadera de ducha</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Regadera + mezclador monocontrol cromado (agua fría/caliente), sistema ahorrador.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ducha accesible (con barras)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ducha a nivel sin sardinel, asiento abatible y barras de apoyo en acero inoxidable (NTC 6047 accesibilidad).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lavamanos de baño</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lavamanos de porcelana (de incrustar u ovalín), con sifón, desagüe y grifería monocontrol ahorradora.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mampara de baño</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mampara en vidrio templado 8 mm con perfilería en aluminio (NSR-10 Título K).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grifería de lavamanos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Monocontrol cromada, aireador ahorrador.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 por lavamanos.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mezclador de ducha</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Monocontrol empotrado, cartucho cerámico.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Regaderas + ducha accesible.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Juego de incrustaciones por baño</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Toallero, jabonera, portarrollos y gancho, en porcelana o acero inoxidable.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">jg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 juego por baño (= N° de sanitarios).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sifón de piso 3" con rejilla</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PVC sanitario + rejilla en acero inoxidable.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mínimo 1 por ducha; agregar los de cocina/zona de ropas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EQUIPO DE ASCENSOR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10.1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ascensor de pasajeros</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ascensor eléctrico sin cuarto de máquinas (MRL), capacidad y paradas POR DEFINIR (6 niveles), NTC 5926 / EN 81-20. Incluye cabina, puertas de piso, guías, contrapeso y control.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gl</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QA crítico: el ascensor no está modelado en Revit. El foso de EST-02 tiene luz libre 1.50 × 1.90 m: validar con el proveedor.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SUPUESTOS Y PARÁMETROS DE CÁLCULO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Celdas en azul con fondo amarillo = parámetros editables. Al cambiarlos se recalculan todas las cantidades derivadas. Fuente indicada en la columna D.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parámetro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuente / criterio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peso nominal barra #3 (3/8")</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kg/m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NSR-10 / NTC 2289</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peso nominal barra #4 (1/2")</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Desperdicio acero de refuerzo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Criterio usual de obra (traslapos y cortes)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Desperdicio concreto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Criterio usual de obra</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unidades de mampostería por m² (bloque arcilla 10×20×30 cm, junta 1 cm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">un/m²</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1/(0.31×0.21). AJUSTAR si la unidad especificada es otra (p.ej. tolete 6×12×24 ≈ 54 un/m² en soga)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Desperdicio unidades de mampostería</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mortero de pega por m² de muro (bloque e=10 cm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">m³/m²</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rendimiento de referencia; ajustar según unidad y espesor de junta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Caras de pañete/estuco/pintura por muro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">caras</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Supuesto: todos los muros se revocan por ambas caras (bruto, sin descontar enchapes)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Espesor de alistado (mortero de nivelación) de piso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Supuesto de diseño; confirmar con nivel de acabado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sobreancho de excavación por lado (foso)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Espacio de trabajo para formaleta exterior</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Profundidad de excavación foso (desde N-0.10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N-0.10 a N-1.50 (EST-02) + 0.05 de solado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Factor de expansión del suelo (sobrantes)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Criterio usual para material común</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Espesor solado de limpieza</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recomendado bajo losa en contacto con suelo (no dibujado en EST-02)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sobreancho solado por lado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Criterio usual</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Densidad acero estructural</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kg/m³</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valor estándar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peso perfil HE 200 (se asume HEB 200)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HEB 200 = 61.3 kg/m; si es HEA 200 usar 42.3 kg/m. EST-02 no lo precisa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Apoyo de dintel por lado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Criterio usual en mampostería</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recubrimiento de impermeabilización interior foso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 = incluir (recomendado para foso bajo nivel de piso)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DATOS DE ENTRADA — EXTRAÍDOS DEL MODELO REVIT (MULTIF H - RVT.rvt)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuente: dashboard index.html (consulta directa al modelo). Solo niveles P1–P5 terminados; P6/P7 y cubierta en diseño, NO incluidos.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. SUPERFICIES Y MUROS POR NIVEL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Concepto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Área cubierta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Programa de superficies Revit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Área exterior</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solo P1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N° de muros de mampostería</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Área de muros de mampostería (neta, una cara)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Revit descuenta vanos de puertas/ventanas. Sin guardaescoba</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. PUERTAS — por función y medida</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Función</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ancho (m)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alto (m)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta de garaje</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta principal de acceso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta de acceso secundario</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Medida imperial 3'×7'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta corrediza social (balcón)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta corrediza de habitación/closet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta corrediza de baño/closet menor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta batiente de habitación</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta batiente de baño/closet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta principal de apartamento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta-ventanal corrediza (balcón)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Puerta corrediza de vestier (herraje Häfele)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Revit reporta ≈7.73 m² de hoja; sin ancho/alto definido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL PUERTAS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. VENTANAS Y VENTANALES — por función y medida</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ventana de habitación</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ventana de baño/cocina</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ventanal de circulación (hall/escalera)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Panel de muro cortina</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ventanal de fachada — acceso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL VENTANAS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. APARATOS SANITARIOS — verificados elemento por elemento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aparato</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL APARATOS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MEMORIA DE CÁLCULO — FOSO DE ASCENSOR (plano EST-02, versión 01, 19/06/2026)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diseño estructural: A3 Ingeniería. Escala 1:25. Cotas en m. Valores en azul tomados del plano; las cantidades son fórmulas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A. GEOMETRÍA (según planta, cortes A-A y B-B)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dato</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luz libre interior del foso — sentido X</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Planta foso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luz libre interior del foso — sentido Y</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Espesor muros de concreto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Planta foso: Muro e=0.15m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lado columna cuadrada (4 und, en esquinas)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Columna 40×40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Número de columnas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Distancia libre entre caras de columnas — X</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Distancia libre entre caras de columnas — Y</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Altura total foso (N-0.10 a N-1.50)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cortes A-A / B-B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Espesor losa de fondo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Losa e=0.20m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Losa — dimensión exterior X (luz + 2 muros)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Losa — dimensión exterior Y (luz + 2 muros)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Huella total con columnas — X</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Huella total con columnas — Y</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Traslapo columna–losa por esquina (lado)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Altura libre muros (sobre losa)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Profundidad útil del foso (N-0.10 a cara superior losa)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Verificar contra la ficha técnica del ascensor elegido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">B. CONCRETO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Elemento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cant.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cálculo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Columnas 40×40 (altura total foso)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4 × 0.40 × 0.40 × 1.40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Losa de fondo e=0.20 (descontando columnas)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.80 × 2.20 × 0.20 − 4 × 0.25² × 0.20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Muros e=0.15 (entre columnas, sobre losa)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(2×1.30 + 2×1.70) × 1.20 × 0.15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solado de limpieza (concreto pobre)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(1.80+0.20) × (2.20+0.20) × 0.05 — recomendado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL CONCRETO ESTRUCTURAL (sin desperdicio)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C. MOVIMIENTO DE TIERRA Y FORMALETA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Excavación manual</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(2.10+0.60) × (2.50+0.60) × 1.45</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Volumen ocupado por el foso + solado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Huella real (losa + salientes de columnas) × 1.40 + solado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Relleno compactado perimetral (material seleccionado)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Excavación − volumen ocupado. Compactar en capas ≤ 0.20 m</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Retiro de sobrantes (suelto)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(Excavación − relleno) × factor de expansión</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Formaleta muros — cara interior</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Perímetro interior 6.80 × 1.20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Formaleta muros — cara exterior</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tramos entre columnas 6.00 × 1.40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Formaleta columnas — caras exteriores expuestas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4 × (2×0.40 + 2×0.15) × 1.40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL FORMALETA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Impermeabilización interior (fondo + muros)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.50×1.90 + 6.80×1.20 — no especificado en EST-02, recomendado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D. CARTILLA DE DESPIECE — ACERO DE REFUERZO fy = 420 MPa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Elemento / posición</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Barra</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Separación (m)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Long. a distribuir (m)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N° barras por capa/elem.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Capas o elementos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N° barras total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">L barra (m)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Long. total (m)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peso (kg)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fuente en plano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Losa fondo — barras sentido X (corto)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corte A-A: recto 1.70 + gancho 180° de 0.20 en cada extremo, L=2.20 (doble parrilla)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Losa fondo — barras sentido Y (largo)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corte B-B: recto 2.10 + gancho 180° de 0.20 en cada extremo, L=2.60 (doble parrilla)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Muros sentido X — horizontales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Planta refuerzo: recto 1.68 + patas a 90° de 0.20, L=2.10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Muros sentido Y — horizontales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Planta refuerzo: recto 2.08 + patas a 90° de 0.20, L=2.50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Muros sentido X — verticales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cortes: recto 1.28 + gancho sup. 180° de 0.20 + pata inf. 90° de 0.20, L=1.75</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Muros sentido Y — verticales</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Columnas 40×40 — longitudinal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirmado: 4 #4 por columna, recto 1.32 + gancho sup. 180° de 0.20 + pata inf. 90° de 0.20, L=1.80</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Columnas 40×40 — flejes cerrados</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirmado: fleje #3 @0.075 L=1.50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subtotal #4 (sin desperdicio)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Subtotal #3 (sin desperdicio)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cuantía de referencia (kg acero / m³ concreto)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E. ESTRUCTURA METÁLICA — DETALLE CONEXIÓN 1 (perfil HE 200 a columna 40×40)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Especificación / cálculo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Platina base A36 300×300×16 mm — unidades</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1 por columna</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Platina base A36 300×300×16 mm — peso</t>
   </si>
   <si>
     <t xml:space="preserve">0.30 × 0.30 × 0.016 × 7850 por platina</t>
@@ -2326,8 +2329,8 @@
         <v>24</v>
       </c>
       <c r="B13" s="6" t="n">
-        <f aca="false">('Foso ascensor'!K53+'Foso ascensor'!K54)*(1+Supuestos!$B$6)</f>
-        <v>342.9657</v>
+        <f aca="false">('Foso ascensor'!I53+'Foso ascensor'!I54)*(1+Supuestos!$B$6)</f>
+        <v>400.05</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>25</v>
@@ -2718,25 +2721,25 @@
       <c r="H14" s="5"/>
       <c r="I14" s="5"/>
       <c r="J14" s="10" t="n">
-        <f aca="false">'Foso ascensor'!K53*(1+Supuestos!$B$6)</f>
-        <v>272.4057</v>
+        <f aca="false">'Foso ascensor'!I53*(1+Supuestos!$B$6)</f>
+        <v>274.05</v>
       </c>
       <c r="K14" s="11" t="s">
         <v>58</v>
       </c>
       <c r="L14" s="5" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>25</v>
@@ -2747,25 +2750,25 @@
       <c r="H15" s="5"/>
       <c r="I15" s="5"/>
       <c r="J15" s="10" t="n">
-        <f aca="false">'Foso ascensor'!K54*(1+Supuestos!$B$6)</f>
-        <v>70.56</v>
+        <f aca="false">'Foso ascensor'!I54*(1+Supuestos!$B$6)</f>
+        <v>126</v>
       </c>
       <c r="K15" s="11" t="s">
         <v>58</v>
       </c>
       <c r="L15" s="5" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>7</v>
@@ -2786,13 +2789,13 @@
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>7</v>
@@ -2807,21 +2810,21 @@
         <v>11.01</v>
       </c>
       <c r="K17" s="11" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="L17" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>22</v>
@@ -2842,13 +2845,13 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>22</v>
@@ -2866,18 +2869,18 @@
         <v>62</v>
       </c>
       <c r="L19" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>15</v>
@@ -2895,18 +2898,18 @@
         <v>51</v>
       </c>
       <c r="L20" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>15</v>
@@ -2927,16 +2930,16 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>106</v>
+        <v>25</v>
       </c>
       <c r="E22" s="5"/>
       <c r="F22" s="5"/>
@@ -3248,7 +3251,7 @@
         <v>139</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>106</v>
+        <v>25</v>
       </c>
       <c r="E31" s="6" t="n">
         <f aca="false">SUMPRODUCT(('Datos Revit'!$B$13:$B$23+2*Supuestos!$B$20),'Datos Revit'!D$13:D$23)+SUMPRODUCT(('Datos Revit'!$B$29:$B$32+2*Supuestos!$B$20),'Datos Revit'!D$29:D$32)</f>
@@ -4338,7 +4341,7 @@
         <v>220</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>106</v>
+        <v>25</v>
       </c>
       <c r="E59" s="6" t="n">
         <f aca="false">SUMPRODUCT('Datos Revit'!$B$29:$B$30,'Datos Revit'!D$29:D$30)</f>
@@ -4857,7 +4860,7 @@
         <v>1</v>
       </c>
       <c r="K72" s="11" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="L72" s="5" t="s">
         <v>265</v>
@@ -7768,10 +7771,10 @@
         <v>45.216</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>25</v>
+        <v>445</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E60" s="2"/>
       <c r="F60" s="2"/>
@@ -7784,7 +7787,7 @@
     </row>
     <row r="61" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B61" s="37" t="n">
         <f aca="false">4*$B$10</f>
@@ -7794,7 +7797,7 @@
         <v>15</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E61" s="2"/>
       <c r="F61" s="2"/>
@@ -7807,17 +7810,17 @@
     </row>
     <row r="62" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="5" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="B62" s="18" t="n">
         <f aca="false">$B$10*1.15</f>
         <v>4.6</v>
       </c>
       <c r="C62" s="5" t="s">
-        <v>106</v>
+        <v>25</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E62" s="2"/>
       <c r="F62" s="2"/>
@@ -7830,7 +7833,7 @@
     </row>
     <row r="63" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="5" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B63" s="37" t="n">
         <f aca="false">$B$10</f>
@@ -7840,7 +7843,7 @@
         <v>15</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E63" s="2"/>
       <c r="F63" s="2"/>
@@ -7878,7 +7881,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -7892,16 +7895,16 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7909,13 +7912,13 @@
         <v>1</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7923,13 +7926,13 @@
         <v>2</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7937,13 +7940,13 @@
         <v>3</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7951,13 +7954,13 @@
         <v>4</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7965,13 +7968,13 @@
         <v>5</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7979,13 +7982,13 @@
         <v>6</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7993,13 +7996,13 @@
         <v>7</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="C10" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>471</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>470</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8007,13 +8010,13 @@
         <v>8</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8021,13 +8024,13 @@
         <v>9</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8035,13 +8038,13 @@
         <v>10</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8049,13 +8052,13 @@
         <v>11</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8063,13 +8066,13 @@
         <v>12</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8077,13 +8080,13 @@
         <v>13</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Foso: conteo de barras según la revisión de obra
Sin barra adicional en los extremos (L1 22, L2 18, M3 14, M4 18) y
flejes solo en 1.20 m sobre la losa (16 por columna, 64 en total).
#4 = 244.40 ml, #3 = 96.00 ml. Compra con inventario: 31 #4 + 17 #3.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGm1Wo5xdbH6HEAejZfCqA
</commit_message>
<xml_diff>
--- a/cantidades/Cantidades_Multifamiliar_Herrera.xlsx
+++ b/cantidades/Cantidades_Multifamiliar_Herrera.xlsx
@@ -1338,7 +1338,7 @@
     <t xml:space="preserve">#3</t>
   </si>
   <si>
-    <t xml:space="preserve">Confirmado: fleje #3 @0.075 L=1.50</t>
+    <t xml:space="preserve">Revisión de obra: fleje #3 @0.075 en 1.20 m sobre la losa, 16 por columna, L=1.50</t>
   </si>
   <si>
     <t xml:space="preserve">Subtotal #4 (sin desperdicio)</t>
@@ -2330,7 +2330,7 @@
       </c>
       <c r="B13" s="6" t="n">
         <f aca="false">('Foso ascensor'!I53+'Foso ascensor'!I54)*(1+Supuestos!$B$6)</f>
-        <v>400.05</v>
+        <v>357.42</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>25</v>
@@ -2722,7 +2722,7 @@
       <c r="I14" s="5"/>
       <c r="J14" s="10" t="n">
         <f aca="false">'Foso ascensor'!I53*(1+Supuestos!$B$6)</f>
-        <v>274.05</v>
+        <v>256.62</v>
       </c>
       <c r="K14" s="11" t="s">
         <v>58</v>
@@ -2751,7 +2751,7 @@
       <c r="I15" s="5"/>
       <c r="J15" s="10" t="n">
         <f aca="false">'Foso ascensor'!I54*(1+Supuestos!$B$6)</f>
-        <v>126</v>
+        <v>100.8</v>
       </c>
       <c r="K15" s="11" t="s">
         <v>58</v>
@@ -7294,22 +7294,22 @@
         <v>2.08</v>
       </c>
       <c r="E45" s="37" t="n">
-        <f aca="false">ROUNDUP(D45/C45,0)+1</f>
-        <v>12</v>
+        <f aca="false">ROUNDUP(D45/C45,0)</f>
+        <v>11</v>
       </c>
       <c r="F45" s="25" t="n">
         <v>2</v>
       </c>
       <c r="G45" s="37" t="n">
         <f aca="false">E45*F45</f>
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="H45" s="29" t="n">
         <v>2.2</v>
       </c>
       <c r="I45" s="18" t="n">
         <f aca="false">G45*H45</f>
-        <v>52.8</v>
+        <v>48.4</v>
       </c>
       <c r="J45" s="38" t="n">
         <f aca="false">Supuestos!$B$5</f>
@@ -7317,7 +7317,7 @@
       </c>
       <c r="K45" s="18" t="n">
         <f aca="false">I45*J45</f>
-        <v>52.4832</v>
+        <v>48.1096</v>
       </c>
       <c r="L45" s="5" t="s">
         <v>422</v>
@@ -7337,22 +7337,22 @@
         <v>1.68</v>
       </c>
       <c r="E46" s="37" t="n">
-        <f aca="false">ROUNDUP(D46/C46,0)+1</f>
-        <v>10</v>
+        <f aca="false">ROUNDUP(D46/C46,0)</f>
+        <v>9</v>
       </c>
       <c r="F46" s="25" t="n">
         <v>2</v>
       </c>
       <c r="G46" s="37" t="n">
         <f aca="false">E46*F46</f>
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H46" s="29" t="n">
         <v>2.6</v>
       </c>
       <c r="I46" s="18" t="n">
         <f aca="false">G46*H46</f>
-        <v>52</v>
+        <v>46.8</v>
       </c>
       <c r="J46" s="38" t="n">
         <f aca="false">Supuestos!$B$5</f>
@@ -7360,7 +7360,7 @@
       </c>
       <c r="K46" s="18" t="n">
         <f aca="false">I46*J46</f>
-        <v>51.688</v>
+        <v>46.5192</v>
       </c>
       <c r="L46" s="5" t="s">
         <v>424</v>
@@ -7380,8 +7380,7 @@
         <f aca="false">$B$20</f>
         <v>1.2</v>
       </c>
-      <c r="E47" s="37" t="n">
-        <f aca="false">ROUNDUP(D47/C47,0)+1</f>
+      <c r="E47" s="25" t="n">
         <v>7</v>
       </c>
       <c r="F47" s="25" t="n">
@@ -7424,8 +7423,7 @@
         <f aca="false">$B$20</f>
         <v>1.2</v>
       </c>
-      <c r="E48" s="37" t="n">
-        <f aca="false">ROUNDUP(D48/C48,0)+1</f>
+      <c r="E48" s="25" t="n">
         <v>7</v>
       </c>
       <c r="F48" s="25" t="n">
@@ -7469,22 +7467,22 @@
         <v>1.3</v>
       </c>
       <c r="E49" s="37" t="n">
-        <f aca="false">ROUNDUP(D49/C49,0)+1</f>
-        <v>8</v>
+        <f aca="false">ROUNDUP(D49/C49,0)</f>
+        <v>7</v>
       </c>
       <c r="F49" s="25" t="n">
         <v>2</v>
       </c>
       <c r="G49" s="37" t="n">
         <f aca="false">E49*F49</f>
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H49" s="29" t="n">
         <v>1.75</v>
       </c>
       <c r="I49" s="18" t="n">
         <f aca="false">G49*H49</f>
-        <v>28</v>
+        <v>24.5</v>
       </c>
       <c r="J49" s="38" t="n">
         <f aca="false">Supuestos!$B$5</f>
@@ -7492,7 +7490,7 @@
       </c>
       <c r="K49" s="18" t="n">
         <f aca="false">I49*J49</f>
-        <v>27.832</v>
+        <v>24.353</v>
       </c>
       <c r="L49" s="5" t="s">
         <v>430</v>
@@ -7513,22 +7511,22 @@
         <v>1.7</v>
       </c>
       <c r="E50" s="37" t="n">
-        <f aca="false">ROUNDUP(D50/C50,0)+1</f>
-        <v>10</v>
+        <f aca="false">ROUNDUP(D50/C50,0)</f>
+        <v>9</v>
       </c>
       <c r="F50" s="25" t="n">
         <v>2</v>
       </c>
       <c r="G50" s="37" t="n">
         <f aca="false">E50*F50</f>
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="H50" s="29" t="n">
         <v>1.75</v>
       </c>
       <c r="I50" s="18" t="n">
         <f aca="false">G50*H50</f>
-        <v>35</v>
+        <v>31.5</v>
       </c>
       <c r="J50" s="38" t="n">
         <f aca="false">Supuestos!$B$5</f>
@@ -7536,7 +7534,7 @@
       </c>
       <c r="K50" s="18" t="n">
         <f aca="false">I50*J50</f>
-        <v>34.79</v>
+        <v>31.311</v>
       </c>
       <c r="L50" s="5" t="s">
         <v>430</v>
@@ -7580,7 +7578,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
         <v>434</v>
       </c>
@@ -7591,26 +7589,26 @@
         <v>0.075</v>
       </c>
       <c r="D52" s="31" t="n">
-        <f aca="false">$B$13</f>
-        <v>1.4</v>
+        <f aca="false">$B$20</f>
+        <v>1.2</v>
       </c>
       <c r="E52" s="37" t="n">
-        <f aca="false">ROUNDUP(D52/C52,0)+1</f>
-        <v>20</v>
+        <f aca="false">ROUNDUP(D52/C52,0)</f>
+        <v>16</v>
       </c>
       <c r="F52" s="25" t="n">
         <v>4</v>
       </c>
       <c r="G52" s="37" t="n">
         <f aca="false">E52*F52</f>
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="H52" s="29" t="n">
         <v>1.5</v>
       </c>
       <c r="I52" s="18" t="n">
         <f aca="false">G52*H52</f>
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="J52" s="38" t="n">
         <f aca="false">Supuestos!$B$4</f>
@@ -7618,7 +7616,7 @@
       </c>
       <c r="K52" s="18" t="n">
         <f aca="false">I52*J52</f>
-        <v>67.2</v>
+        <v>53.76</v>
       </c>
       <c r="L52" s="5" t="s">
         <v>436</v>
@@ -7637,12 +7635,12 @@
       <c r="H53" s="2"/>
       <c r="I53" s="36" t="n">
         <f aca="false">SUMIF(B45:B52,"#4",I45:I52)</f>
-        <v>261</v>
+        <v>244.4</v>
       </c>
       <c r="J53" s="2"/>
       <c r="K53" s="36" t="n">
         <f aca="false">SUMIF(B45:B52,"#4",K45:K52)</f>
-        <v>259.434</v>
+        <v>242.9336</v>
       </c>
       <c r="L53" s="2"/>
     </row>
@@ -7659,12 +7657,12 @@
       <c r="H54" s="2"/>
       <c r="I54" s="36" t="n">
         <f aca="false">SUMIF(B45:B52,"#3",I45:I52)</f>
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="J54" s="2"/>
       <c r="K54" s="36" t="n">
         <f aca="false">SUMIF(B45:B52,"#3",K45:K52)</f>
-        <v>67.2</v>
+        <v>53.76</v>
       </c>
       <c r="L54" s="2"/>
     </row>
@@ -7683,7 +7681,7 @@
       <c r="J55" s="2"/>
       <c r="K55" s="40" t="n">
         <f aca="false">(K53+K54)/B29</f>
-        <v>120.174392935982</v>
+        <v>109.158793230316</v>
       </c>
       <c r="L55" s="2"/>
     </row>

</xml_diff>

<commit_message>
Foso: solado de limpieza cubre también las columnas (2.70 × 2.30 m)
El concreto estructural se verificó con un conteo independiente: 2.718 m³.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGm1Wo5xdbH6HEAejZfCqA
</commit_message>
<xml_diff>
--- a/cantidades/Cantidades_Multifamiliar_Herrera.xlsx
+++ b/cantidades/Cantidades_Multifamiliar_Herrera.xlsx
@@ -1194,7 +1194,7 @@
     <t xml:space="preserve">Solado de limpieza (concreto pobre)</t>
   </si>
   <si>
-    <t xml:space="preserve">(1.80+0.20) × (2.20+0.20) × 0.05 — recomendado</t>
+    <t xml:space="preserve">(2.10+0.20) × (2.50+0.20) × 0.05: bajo losa y columnas — recomendado</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL CONCRETO ESTRUCTURAL (sin desperdicio)</t>
@@ -2606,7 +2606,7 @@
       <c r="I10" s="5"/>
       <c r="J10" s="12" t="n">
         <f aca="false">'Foso ascensor'!B28*(1+Supuestos!$B$7)</f>
-        <v>0.252</v>
+        <v>0.326025</v>
       </c>
       <c r="K10" s="11" t="s">
         <v>62</v>
@@ -2836,7 +2836,7 @@
       <c r="I18" s="5"/>
       <c r="J18" s="10" t="n">
         <f aca="false">'Foso ascensor'!B35</f>
-        <v>5.8065</v>
+        <v>5.736</v>
       </c>
       <c r="K18" s="11" t="s">
         <v>62</v>
@@ -2863,7 +2863,7 @@
       <c r="I19" s="5"/>
       <c r="J19" s="10" t="n">
         <f aca="false">'Foso ascensor'!B36</f>
-        <v>8.229</v>
+        <v>8.32065</v>
       </c>
       <c r="K19" s="11" t="s">
         <v>62</v>
@@ -6911,13 +6911,13 @@
       <c r="K27" s="2"/>
       <c r="L27" s="2"/>
     </row>
-    <row r="28" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
         <v>387</v>
       </c>
       <c r="B28" s="33" t="n">
-        <f aca="false">($B$15+2*Supuestos!$B$17)*($B$16+2*Supuestos!$B$17)*Supuestos!$B$16</f>
-        <v>0.24</v>
+        <f aca="false">($B$17+2*Supuestos!$B$17)*($B$18+2*Supuestos!$B$17)*Supuestos!$B$16</f>
+        <v>0.3105</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>22</v>
@@ -7036,7 +7036,7 @@
       </c>
       <c r="B34" s="18" t="n">
         <f aca="false">($B$15*$B$16+$B$10*($B$9^2-$B$19^2))*$B$13+B28</f>
-        <v>6.33</v>
+        <v>6.4005</v>
       </c>
       <c r="C34" s="5" t="s">
         <v>22</v>
@@ -7059,7 +7059,7 @@
       </c>
       <c r="B35" s="18" t="n">
         <f aca="false">B33-B34</f>
-        <v>5.8065</v>
+        <v>5.736</v>
       </c>
       <c r="C35" s="5" t="s">
         <v>22</v>
@@ -7082,7 +7082,7 @@
       </c>
       <c r="B36" s="18" t="n">
         <f aca="false">(B33-B35)*Supuestos!$B$15</f>
-        <v>8.229</v>
+        <v>8.32065</v>
       </c>
       <c r="C36" s="5" t="s">
         <v>22</v>

</xml_diff>